<commit_message>
Schema overrides per project, --optional flag for audits, dashboard polish and screenshot
</commit_message>
<xml_diff>
--- a/data/output/samples/seed_companies_audit.xlsx
+++ b/data/output/samples/seed_companies_audit.xlsx
@@ -1243,7 +1243,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-08 08:51</t>
+          <t>2026-09-08 09:01</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="Y2" s="14" t="n">
-        <v>34.8</v>
+        <v>36.4</v>
       </c>
       <c r="Z2" s="13" t="inlineStr">
         <is>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="AH2" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI2" s="11" t="n"/>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="X3" s="13" t="n"/>
       <c r="Y3" s="14" t="n">
-        <v>26.1</v>
+        <v>27.3</v>
       </c>
       <c r="Z3" s="13" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
       <c r="AG3" s="11" t="n"/>
       <c r="AH3" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI3" s="11" t="n"/>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="X4" s="13" t="n"/>
       <c r="Y4" s="14" t="n">
-        <v>30.4</v>
+        <v>31.8</v>
       </c>
       <c r="Z4" s="13" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
       <c r="AG4" s="11" t="n"/>
       <c r="AH4" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI4" s="11" t="n"/>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="X5" s="13" t="n"/>
       <c r="Y5" s="14" t="n">
-        <v>34.8</v>
+        <v>36.4</v>
       </c>
       <c r="Z5" s="13" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
       <c r="AG5" s="11" t="n"/>
       <c r="AH5" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI5" s="11" t="n"/>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="X6" s="13" t="n"/>
       <c r="Y6" s="14" t="n">
-        <v>26.1</v>
+        <v>27.3</v>
       </c>
       <c r="Z6" s="13" t="inlineStr">
         <is>
@@ -2054,7 +2054,7 @@
       <c r="AG6" s="11" t="n"/>
       <c r="AH6" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI6" s="11" t="n"/>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="X7" s="13" t="n"/>
       <c r="Y7" s="14" t="n">
-        <v>21.7</v>
+        <v>22.7</v>
       </c>
       <c r="Z7" s="13" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
       <c r="AG7" s="11" t="n"/>
       <c r="AH7" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI7" s="11" t="n"/>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="X8" s="13" t="n"/>
       <c r="Y8" s="14" t="n">
-        <v>30.4</v>
+        <v>31.8</v>
       </c>
       <c r="Z8" s="13" t="inlineStr">
         <is>
@@ -2246,7 +2246,7 @@
       <c r="AG8" s="11" t="n"/>
       <c r="AH8" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI8" s="11" t="n"/>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="Y9" s="14" t="n">
-        <v>39.1</v>
+        <v>40.9</v>
       </c>
       <c r="Z9" s="13" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="AH9" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI9" s="11" t="n"/>
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="Y10" s="14" t="n">
-        <v>34.8</v>
+        <v>36.4</v>
       </c>
       <c r="Z10" s="13" t="inlineStr">
         <is>
@@ -2470,7 +2470,7 @@
       <c r="AG10" s="11" t="n"/>
       <c r="AH10" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI10" s="11" t="n"/>
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="Y11" s="14" t="n">
-        <v>39.1</v>
+        <v>40.9</v>
       </c>
       <c r="Z11" s="13" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       <c r="AG11" s="11" t="n"/>
       <c r="AH11" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
       <c r="AI11" s="11" t="n"/>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-08T08:51:45+00:00</t>
+          <t>2026-09-08T09:01:00+00:00</t>
         </is>
       </c>
     </row>
@@ -3449,9 +3449,9 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>required column(s) not present in the file: Category - add them before delivery</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
     </row>
@@ -3499,10 +3499,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
-    <mergeCell ref="A23:E23"/>
     <mergeCell ref="B28:E28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3659,11 +3658,7 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="D5" s="11" t="inlineStr"/>
       <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Main business category (e.g. restaurant, cafe, software company).</t>

</xml_diff>